<commit_message>
Update sample excel templates with exact headers and data from word document
</commit_message>
<xml_diff>
--- a/webapp/public/templates/10. BÁO CÁO BSC_NHI.xlsx
+++ b/webapp/public/templates/10. BÁO CÁO BSC_NHI.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,14 +477,855 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bến Lức</t>
+          <t>1. Tổng doanh thu VT-CNTT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>139.178</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0,00%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Đức Hòa</t>
+          <t>2. Doanh thu cho thuê hạ tầng</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.722</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>206,350</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>154,408</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>141,191</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>141,883</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>568,606</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>202,578</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>124,515</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1.539,530</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. Sử dụng tiết kiệm điện so với cùng kỳ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>98,00%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Hệ số hàng tồn kho</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. TL phiếu xử lý SC đúng hạn CĐ5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>98,00%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>98,06%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>98,42%</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>96,99%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>95,91%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>98,30%</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>98,29%</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>97,44%</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>97,44%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6. Đảm bảo năng lực hạ tầng BRCD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2,00%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0,89%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2,23%</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1,93%</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0,84%</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0,29%</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1,43%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7. TB BRCD/MyTV/TSLC do chất lượng đường dây GPON kém</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0,037%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0,145%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0,219%</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0,431%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0,156%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0,140%</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0,25%</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0,221%</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0,212%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8. Hài lòng KH sau xử lý PAKH về chất lượng mạng di động</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>99,80%</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9. Thuê bao hủy theo mục tiêu</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2280 TB</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>466</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>374</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2546</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10. TB BRCD gián đoạn dịch vụ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0,50%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0,25%</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2,68%</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0,37%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11. Chất lượng hạ tầng VT-CNTT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>99,00%</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>98,48%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>98,27%</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>98,38%</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>98,45%</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>98,39%</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>98,63%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>98,65%</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>98,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12. Thời gian MLL các thiết bị di động  3G/4G/5G</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4,56</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3,93</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>12,44</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6,52</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>9,87</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>4,28</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1,91</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>6,46</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13. Tỉ lệ cung cấp và cấu hình dịch vụ tự động BRCĐ</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>90,00%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>95,90%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>93,40%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>94,66%</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>97,38%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>98,06%</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>92,74%</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>96,17%</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>95,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14. Hoàn thành công việc được giao</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>16. Mức độ tuân thủ quy trình, quy định</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -499,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,14 +1368,198 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bến Lức</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Đức Hòa</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>100,25</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Đức Hòa</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bến Lức</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>99,74</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tân Châu</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>98,74</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tân An</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>97,45</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tân Ninh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>96,78</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tổ Tổng hợp</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>96,74</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tổ Khai thác</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>96,74</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gò Dầu</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>96,23</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kiến Tường</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>95,87</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>

</xml_diff>